<commit_message>
Refresh figures, source data, and experiment code
</commit_message>
<xml_diff>
--- a/data/Figure_6_source_data/Figure_6_loss_data.xlsx
+++ b/data/Figure_6_source_data/Figure_6_loss_data.xlsx
@@ -397,51 +397,62 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:E3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>theta_1_dot</v>
+        <v>Model</v>
       </c>
       <c r="B1" t="str">
-        <v>theta_2_dot</v>
+        <v>Lorenz-96</v>
       </c>
       <c r="C1" t="str">
-        <v>theta_3_dot</v>
+        <v>phi_4</v>
       </c>
       <c r="D1" t="str">
-        <v>theta_1_ddot</v>
+        <v>DNLS</v>
       </c>
       <c r="E1" t="str">
-        <v>theta_2_ddot</v>
-      </c>
-      <c r="F1" t="str">
-        <v>theta3_ddot</v>
+        <v>AL</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2.0E-15</v>
+        <v>Average Loss</v>
       </c>
       <c r="B2" t="str">
-        <v>3.07E-12</v>
+        <v>8.4E-11</v>
       </c>
       <c r="C2" t="str">
-        <v>2.1E-13</v>
+        <v>8.0E-11</v>
       </c>
       <c r="D2" t="str">
-        <v>2.21E-1</v>
+        <v>3.9E-12</v>
       </c>
       <c r="E2" t="str">
-        <v>1.096</v>
-      </c>
-      <c r="F2" t="str">
-        <v>2.904</v>
+        <v>1.7E-11</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Coefficient Error</v>
+      </c>
+      <c r="B3" t="str">
+        <v>3.0E-6</v>
+      </c>
+      <c r="C3" t="str">
+        <v>1.1E-7</v>
+      </c>
+      <c r="D3" t="str">
+        <v>8.5E-8</v>
+      </c>
+      <c r="E3" t="str">
+        <v>7.4E-7</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>